<commit_message>
second Excel activity file
</commit_message>
<xml_diff>
--- a/12603253.xlsx
+++ b/12603253.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kraj5\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5E34081-88A6-4C8E-B216-BEBD9C3BF93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500047D9-D8B1-49AC-A9BD-8EF5062F5CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t xml:space="preserve"> August</t>
+  </si>
+  <si>
+    <t>Neutral</t>
   </si>
 </sst>
 </file>
@@ -1031,25 +1034,47 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15" t="str">
+      <c r="A7" s="8">
+        <v>46223</v>
+      </c>
+      <c r="B7" s="9">
+        <v>420</v>
+      </c>
+      <c r="C7" s="9">
+        <v>45</v>
+      </c>
+      <c r="D7" s="9">
+        <v>120</v>
+      </c>
+      <c r="E7" s="9">
+        <v>90</v>
+      </c>
+      <c r="F7" s="9">
+        <v>180</v>
+      </c>
+      <c r="G7" s="9">
+        <v>3</v>
+      </c>
+      <c r="H7" s="9">
+        <v>30</v>
+      </c>
+      <c r="I7" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="15" t="str">
+        <v>885</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
+        <v>555</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N7" s="17"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>